<commit_message>
Update GUA Waste model files
</commit_message>
<xml_diff>
--- a/GUA/Waste/A1_Inputs/A-I_Horizon_Configuration.xlsx
+++ b/GUA/Waste/A1_Inputs/A-I_Horizon_Configuration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://clgcr.sharepoint.com/sites/ClimateLeadGroup-Decarb_GU/Documentos compartidos/Decarb_GU/4_Model/2_Residuos&amp;PIUP/modelo_waste_202302/t1_confection/A1_Inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IgnacioAlfaroCorrale\Desktop\Models_running\Waste_CR_v4\A1_Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{12A48412-8A79-41A4-8D13-3854B5441106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D43FADD4-E540-4C71-8DBA-B9CF20C31924}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0545BAC-5362-431A-9028-F38369A040C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Horizon" sheetId="1" r:id="rId1"/>
@@ -374,13 +374,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -388,7 +388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>2018</v>
       </c>
@@ -403,6 +403,16 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a1fcbaaf-06d9-47c4-b3a2-beefbc45d784">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -411,7 +421,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000360DE9767CDF0449BF75EAB371D3CB7" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="75cb9a07855af6ac97bd432464ca7c04">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1fcbaaf-06d9-47c4-b3a2-beefbc45d784" xmlns:ns3="081a93ea-d517-42a5-a2b7-457060aa7471" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d1676634304aab9936f6a5a5f53c7423" ns2:_="" ns3:_="">
     <xsd:import namespace="a1fcbaaf-06d9-47c4-b3a2-beefbc45d784"/>
@@ -634,28 +644,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a1fcbaaf-06d9-47c4-b3a2-beefbc45d784">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4E3C48B-2607-4511-AB50-EE5AE65E4E72}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{145250E9-3F72-4934-99AB-D125CBCD5637}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="48eed89a-7418-4977-ae3a-838f0fac8ec5"/>
+    <ds:schemaRef ds:uri="416d42ac-85ec-40c4-8054-6c816fd4b6a7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB815CDD-081E-435E-8A65-3F13801F858B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E425D3D-510D-4789-99BF-6BECF10818E8}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F751D4EF-A311-4CB3-A3BF-B35A3B071594}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{421CE1AF-0B37-451D-9948-2C5A7580DB28}"/>
 </file>
</xml_diff>